<commit_message>
Updated to have inputs via Excel input file - does not work with indexed colors
</commit_message>
<xml_diff>
--- a/Figures.xlsx
+++ b/Figures.xlsx
@@ -41,26 +41,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0083CCEB"/>
-        <bgColor rgb="0083CCEB"/>
+        <fgColor rgb="FF83CCEB"/>
+        <bgColor rgb="FF83CCEB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DAE9F8"/>
-        <bgColor rgb="00DAE9F8"/>
+        <fgColor rgb="FFDAE9F8"/>
+        <bgColor rgb="FFDAE9F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A6C9EC"/>
-        <bgColor rgb="00A6C9EC"/>
+        <fgColor rgb="FFF72727"/>
+        <bgColor rgb="FFF72727"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6C9EC"/>
-        <bgColor rgb="00C6C9EC"/>
+        <fgColor rgb="FFC6C9EC"/>
+        <bgColor rgb="FFC6C9EC"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>

<commit_message>
Updated to fix signage bug. Excel Inputs running into a Permissions Denied bug.
</commit_message>
<xml_diff>
--- a/Figures.xlsx
+++ b/Figures.xlsx
@@ -53,8 +53,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF72727"/>
-        <bgColor rgb="FFF72727"/>
+        <fgColor rgb="FFA6C9EC"/>
+        <bgColor rgb="FFA6C9EC"/>
       </patternFill>
     </fill>
     <fill>

</xml_diff>